<commit_message>
feat(scripts): phase7b-insert-missing-xlsx + sync 30 TCs P2 faltantes en xlsx
Mini-script dedicado para insertar en xlsx los TCs presentes en el JSON
normalizado pero sin fila fisica en STRIPE_Test_Suite_Matriz_Sincronizado.xlsx.
update-matriz-xlsx.ts actualiza filas existentes pero NO inserta.

Fase P3.3: se agregaron 30 TCs (TS-STRIPE-P2-TC060..089 — operaciones
recurrentes/clonacion/edicion) al sheet 'TEST_SUITE 2.0'. Resultado post-sync:
  matched=219, orphans=11 (BUG_REPORT + SMOKE_TESTING esperados), missing=0

Uso: node scripts/ai/phase7b-insert-missing-xlsx.mjs [--apply]

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
+++ b/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3931" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4021" uniqueCount="720">
   <si>
     <t>Feature / Módulo</t>
   </si>
@@ -1634,6 +1634,111 @@
   </si>
   <si>
     <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>gateway-pg-stripe/reactivation</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC060 – Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC061 – Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC062 – Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC063 – Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC064 – Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC065 – Validar Reactivación de viaje cancelado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>gateway-pg-stripe/clone</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC066 – Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC067 – Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC068 – Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC069 – Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC070 – Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC071 – Validar Clonación de viaje cancelado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC072 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC073 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC074 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC075 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC076 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC077 – Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>gateway-pg-stripe/edit</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC078 – Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC079 – Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC080 – Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC081 – Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC082 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC083 – Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC084 – Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC085 – Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC086 – Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC087 – Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC088 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+  </si>
+  <si>
+    <t>TS-STRIPE-P2-TC089 – Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
   </si>
   <si>
     <t>Fuente</t>
@@ -10462,37 +10567,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>675</v>
+        <v>710</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>664</v>
+        <v>699</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>676</v>
+        <v>711</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>666</v>
+        <v>701</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>667</v>
+        <v>702</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>668</v>
+        <v>703</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>669</v>
+        <v>704</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>677</v>
+        <v>712</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>678</v>
+        <v>713</v>
       </c>
       <c r="J1" s="16" t="s">
-        <v>679</v>
+        <v>714</v>
       </c>
       <c r="K1" s="16" t="s">
-        <v>680</v>
+        <v>715</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -10543,7 +10648,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>681</v>
+        <v>716</v>
       </c>
       <c r="B4">
         <v>18</v>
@@ -10589,7 +10694,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>682</v>
+        <v>717</v>
       </c>
       <c r="B6">
         <v>15</v>
@@ -10625,28 +10730,28 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>683</v>
+        <v>718</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>675</v>
+        <v>710</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>657</v>
+        <v>692</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>483</v>
+        <v>518</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>487</v>
+        <v>522</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>684</v>
+        <v>719</v>
       </c>
       <c r="I1" t="s">
         <v>22</v>
@@ -10665,7 +10770,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:X60"/>
+  <dimension ref="A1:X90"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.90625" customHeight="1"/>
   <cols>
     <col min="1" max="22" width="24" customWidth="1"/>
@@ -14402,6 +14507,336 @@
         <v>327</v>
       </c>
       <c r="V60" s="8"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>473</v>
+      </c>
+      <c r="B61" t="s">
+        <v>474</v>
+      </c>
+      <c r="C61" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>473</v>
+      </c>
+      <c r="B62" t="s">
+        <v>476</v>
+      </c>
+      <c r="C62" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>473</v>
+      </c>
+      <c r="B63" t="s">
+        <v>477</v>
+      </c>
+      <c r="C63" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>473</v>
+      </c>
+      <c r="B64" t="s">
+        <v>478</v>
+      </c>
+      <c r="C64" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>473</v>
+      </c>
+      <c r="B65" t="s">
+        <v>479</v>
+      </c>
+      <c r="C65" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>473</v>
+      </c>
+      <c r="B66" t="s">
+        <v>481</v>
+      </c>
+      <c r="C66" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>482</v>
+      </c>
+      <c r="B67" t="s">
+        <v>483</v>
+      </c>
+      <c r="C67" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>482</v>
+      </c>
+      <c r="B68" t="s">
+        <v>484</v>
+      </c>
+      <c r="C68" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>482</v>
+      </c>
+      <c r="B69" t="s">
+        <v>485</v>
+      </c>
+      <c r="C69" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>482</v>
+      </c>
+      <c r="B70" t="s">
+        <v>486</v>
+      </c>
+      <c r="C70" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>482</v>
+      </c>
+      <c r="B71" t="s">
+        <v>487</v>
+      </c>
+      <c r="C71" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>482</v>
+      </c>
+      <c r="B72" t="s">
+        <v>488</v>
+      </c>
+      <c r="C72" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>482</v>
+      </c>
+      <c r="B73" t="s">
+        <v>489</v>
+      </c>
+      <c r="C73" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>482</v>
+      </c>
+      <c r="B74" t="s">
+        <v>490</v>
+      </c>
+      <c r="C74" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>482</v>
+      </c>
+      <c r="B75" t="s">
+        <v>491</v>
+      </c>
+      <c r="C75" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>482</v>
+      </c>
+      <c r="B76" t="s">
+        <v>492</v>
+      </c>
+      <c r="C76" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>482</v>
+      </c>
+      <c r="B77" t="s">
+        <v>493</v>
+      </c>
+      <c r="C77" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>482</v>
+      </c>
+      <c r="B78" t="s">
+        <v>494</v>
+      </c>
+      <c r="C78" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>495</v>
+      </c>
+      <c r="B79" t="s">
+        <v>496</v>
+      </c>
+      <c r="C79" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>495</v>
+      </c>
+      <c r="B80" t="s">
+        <v>497</v>
+      </c>
+      <c r="C80" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>495</v>
+      </c>
+      <c r="B81" t="s">
+        <v>498</v>
+      </c>
+      <c r="C81" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>495</v>
+      </c>
+      <c r="B82" t="s">
+        <v>499</v>
+      </c>
+      <c r="C82" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>495</v>
+      </c>
+      <c r="B83" t="s">
+        <v>500</v>
+      </c>
+      <c r="C83" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>495</v>
+      </c>
+      <c r="B84" t="s">
+        <v>501</v>
+      </c>
+      <c r="C84" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>495</v>
+      </c>
+      <c r="B85" t="s">
+        <v>502</v>
+      </c>
+      <c r="C85" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>495</v>
+      </c>
+      <c r="B86" t="s">
+        <v>503</v>
+      </c>
+      <c r="C86" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>495</v>
+      </c>
+      <c r="B87" t="s">
+        <v>504</v>
+      </c>
+      <c r="C87" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>495</v>
+      </c>
+      <c r="B88" t="s">
+        <v>505</v>
+      </c>
+      <c r="C88" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>495</v>
+      </c>
+      <c r="B89" t="s">
+        <v>506</v>
+      </c>
+      <c r="C89" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>495</v>
+      </c>
+      <c r="B90" t="s">
+        <v>507</v>
+      </c>
+      <c r="C90" t="s">
+        <v>480</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14421,39 +14856,39 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>473</v>
+        <v>508</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>474</v>
+        <v>509</v>
       </c>
     </row>
     <row r="2" ht="28.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>475</v>
+        <v>510</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>476</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" ht="72" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>477</v>
+        <v>512</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" ht="86.4" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>479</v>
+        <v>514</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>480</v>
+        <v>515</v>
       </c>
     </row>
     <row r="5" ht="28.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>481</v>
+        <v>516</v>
       </c>
       <c r="B5" s="8">
         <v>59</v>
@@ -14498,70 +14933,70 @@
   <sheetData>
     <row r="1" ht="28.75" customHeight="1" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>483</v>
+        <v>518</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>484</v>
+        <v>519</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>487</v>
+        <v>522</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>488</v>
+        <v>523</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>489</v>
+        <v>524</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>490</v>
+        <v>525</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>491</v>
+        <v>526</v>
       </c>
       <c r="K1" s="11" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>492</v>
+        <v>527</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="N1" s="11" t="s">
-        <v>494</v>
+        <v>529</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>495</v>
+        <v>530</v>
       </c>
       <c r="P1" s="11" t="s">
-        <v>496</v>
+        <v>531</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>497</v>
+        <v>532</v>
       </c>
       <c r="R1" s="11" t="s">
-        <v>498</v>
+        <v>533</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>499</v>
+        <v>534</v>
       </c>
       <c r="T1" s="11" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="U1" s="11" t="s">
-        <v>501</v>
+        <v>536</v>
       </c>
       <c r="V1" s="11" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="W1" s="10" t="s">
         <v>22</v>
@@ -14572,13 +15007,13 @@
     </row>
     <row r="2" ht="244.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>503</v>
+        <v>538</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>504</v>
+        <v>539</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>505</v>
+        <v>540</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>30</v>
@@ -14587,36 +15022,36 @@
         <v>30</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>507</v>
+        <v>542</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>508</v>
+        <v>543</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>510</v>
+        <v>545</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>511</v>
+        <v>546</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>512</v>
+        <v>547</v>
       </c>
     </row>
     <row r="3" ht="409.6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>513</v>
+        <v>548</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>514</v>
+        <v>549</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>515</v>
+        <v>550</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>29</v>
@@ -14628,22 +15063,22 @@
         <v>61</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>517</v>
+        <v>552</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>518</v>
+        <v>553</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>519</v>
+        <v>554</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>520</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -14669,25 +15104,25 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>521</v>
+        <v>556</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>522</v>
+        <v>557</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>523</v>
+        <v>558</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>524</v>
+        <v>559</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>525</v>
+        <v>560</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>526</v>
+        <v>561</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>527</v>
+        <v>562</v>
       </c>
       <c r="H1" t="s">
         <v>22</v>
@@ -14701,22 +15136,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>528</v>
+        <v>563</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>529</v>
+        <v>564</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>530</v>
+        <v>565</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -14724,22 +15159,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>533</v>
+        <v>568</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>534</v>
+        <v>569</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>535</v>
+        <v>570</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -14747,22 +15182,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>536</v>
+        <v>571</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>537</v>
+        <v>572</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>538</v>
+        <v>573</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -14770,22 +15205,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>539</v>
+        <v>574</v>
       </c>
       <c r="C5" t="s">
-        <v>540</v>
+        <v>575</v>
       </c>
       <c r="D5" t="s">
-        <v>541</v>
+        <v>576</v>
       </c>
       <c r="E5" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F5" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G5" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -14793,22 +15228,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>544</v>
+        <v>579</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>545</v>
+        <v>580</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>546</v>
+        <v>581</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -14816,22 +15251,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>547</v>
+        <v>582</v>
       </c>
       <c r="C7" t="s">
-        <v>548</v>
+        <v>583</v>
       </c>
       <c r="D7" t="s">
-        <v>549</v>
+        <v>584</v>
       </c>
       <c r="E7" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F7" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G7" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -14839,22 +15274,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>550</v>
+        <v>585</v>
       </c>
       <c r="C8" t="s">
-        <v>551</v>
+        <v>586</v>
       </c>
       <c r="D8" t="s">
-        <v>552</v>
+        <v>587</v>
       </c>
       <c r="E8" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F8" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G8" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -14862,22 +15297,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>553</v>
+        <v>588</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>554</v>
+        <v>589</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>555</v>
+        <v>590</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -14885,22 +15320,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="C10" t="s">
-        <v>557</v>
+        <v>592</v>
       </c>
       <c r="D10" t="s">
-        <v>558</v>
+        <v>593</v>
       </c>
       <c r="E10" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="F10" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G10" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
     </row>
   </sheetData>
@@ -14930,386 +15365,386 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>559</v>
+        <v>594</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>560</v>
+        <v>595</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>561</v>
+        <v>596</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>562</v>
+        <v>597</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>563</v>
+        <v>598</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>564</v>
+        <v>599</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>565</v>
+        <v>600</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>566</v>
+        <v>601</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>567</v>
+        <v>602</v>
       </c>
     </row>
     <row r="2" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>568</v>
+        <v>603</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>569</v>
+        <v>604</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>570</v>
+        <v>605</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>569</v>
+        <v>604</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>569</v>
+        <v>604</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>569</v>
+        <v>604</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>571</v>
+        <v>606</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>530</v>
+        <v>565</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="3" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>572</v>
+        <v>607</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>576</v>
+        <v>611</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>577</v>
+        <v>612</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>578</v>
+        <v>613</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>579</v>
+        <v>614</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="4" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>572</v>
+        <v>607</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>576</v>
+        <v>611</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>580</v>
+        <v>615</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>581</v>
+        <v>616</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>582</v>
+        <v>617</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
     </row>
     <row r="5" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>583</v>
+        <v>618</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>584</v>
+        <v>619</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>586</v>
+        <v>621</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>587</v>
+        <v>622</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
     </row>
     <row r="6" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>583</v>
+        <v>618</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>584</v>
+        <v>619</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>576</v>
+        <v>611</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>586</v>
+        <v>621</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>589</v>
+        <v>624</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>590</v>
+        <v>625</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="7" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>583</v>
+        <v>618</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>584</v>
+        <v>619</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>591</v>
+        <v>626</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>592</v>
+        <v>627</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>593</v>
+        <v>628</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>594</v>
+        <v>629</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="8" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>583</v>
+        <v>618</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>584</v>
+        <v>619</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>591</v>
+        <v>626</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>595</v>
+        <v>630</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>596</v>
+        <v>631</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>597</v>
+        <v>632</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>598</v>
+        <v>633</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>599</v>
+        <v>634</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>600</v>
+        <v>635</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>601</v>
+        <v>636</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>602</v>
+        <v>637</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>603</v>
+        <v>638</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="10" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>598</v>
+        <v>633</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>599</v>
+        <v>634</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>600</v>
+        <v>635</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>592</v>
+        <v>627</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>604</v>
+        <v>639</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>605</v>
+        <v>640</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="11" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>598</v>
+        <v>633</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>599</v>
+        <v>634</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>600</v>
+        <v>635</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>606</v>
+        <v>641</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>607</v>
+        <v>642</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>608</v>
+        <v>643</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
     </row>
     <row r="12" ht="29" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>609</v>
+        <v>644</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>609</v>
+        <v>644</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>610</v>
+        <v>645</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>611</v>
+        <v>646</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>601</v>
+        <v>636</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>613</v>
+        <v>648</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>614</v>
+        <v>649</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -15333,142 +15768,142 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>615</v>
+        <v>650</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>616</v>
+        <v>651</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>617</v>
+        <v>652</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>566</v>
+        <v>601</v>
       </c>
     </row>
     <row r="2" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>618</v>
+        <v>653</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>619</v>
+        <v>654</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>620</v>
+        <v>655</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>530</v>
+        <v>565</v>
       </c>
     </row>
     <row r="3" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>621</v>
+        <v>656</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>622</v>
+        <v>657</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>623</v>
+        <v>658</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>624</v>
+        <v>659</v>
       </c>
     </row>
     <row r="4" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>625</v>
+        <v>660</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>626</v>
+        <v>661</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>627</v>
+        <v>662</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>628</v>
+        <v>663</v>
       </c>
     </row>
     <row r="5" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>629</v>
+        <v>664</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>630</v>
+        <v>665</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>631</v>
+        <v>666</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>624</v>
+        <v>659</v>
       </c>
     </row>
     <row r="6" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>632</v>
+        <v>667</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>633</v>
+        <v>668</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>634</v>
+        <v>669</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>635</v>
+        <v>670</v>
       </c>
     </row>
     <row r="7" ht="43.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>636</v>
+        <v>671</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>637</v>
+        <v>672</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>638</v>
+        <v>673</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>639</v>
+        <v>674</v>
       </c>
     </row>
     <row r="8" ht="72.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>640</v>
+        <v>675</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>641</v>
+        <v>676</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>642</v>
+        <v>677</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>643</v>
+        <v>678</v>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>644</v>
+        <v>679</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>645</v>
+        <v>680</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>647</v>
+        <v>682</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>648</v>
+        <v>683</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>649</v>
+        <v>684</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>650</v>
+        <v>685</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>651</v>
+        <v>686</v>
       </c>
     </row>
   </sheetData>
@@ -15486,43 +15921,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>652</v>
+        <v>687</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>653</v>
+        <v>688</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>654</v>
+        <v>689</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>489</v>
+        <v>524</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>655</v>
+        <v>690</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>656</v>
+        <v>691</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>657</v>
+        <v>692</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>658</v>
+        <v>693</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="J1" s="16" t="s">
-        <v>494</v>
+        <v>529</v>
       </c>
       <c r="K1" s="16" t="s">
-        <v>495</v>
+        <v>530</v>
       </c>
       <c r="L1" s="16" t="s">
-        <v>659</v>
+        <v>694</v>
       </c>
       <c r="M1" s="16" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
     </row>
   </sheetData>
@@ -15540,49 +15975,49 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>661</v>
+        <v>696</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>489</v>
+        <v>524</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>662</v>
+        <v>697</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>663</v>
+        <v>698</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>664</v>
+        <v>699</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>665</v>
+        <v>700</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>666</v>
+        <v>701</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>667</v>
+        <v>702</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>668</v>
+        <v>703</v>
       </c>
       <c r="J1" s="16" t="s">
-        <v>669</v>
+        <v>704</v>
       </c>
       <c r="K1" s="16" t="s">
-        <v>670</v>
+        <v>705</v>
       </c>
       <c r="L1" s="16" t="s">
-        <v>671</v>
+        <v>706</v>
       </c>
       <c r="M1" s="16" t="s">
-        <v>672</v>
+        <v>707</v>
       </c>
       <c r="N1" s="16" t="s">
-        <v>673</v>
+        <v>708</v>
       </c>
       <c r="O1" s="16" t="s">
-        <v>674</v>
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync(xlsx): STRIPE_Test_Suite_Matriz_Sincronizado.xlsx tras rename Eje 2
Aplicado via scripts/ai/matriz-coherencia/sync-xlsx-rename-personal.py:
- 128 renames Eje 2 en columnas B (Título) y C (Descripción).
- Preservadas celdas no afectadas, estilos y colores (openpyxl).

Alcance xlsx: solo matriz parte 1 (TS-STRIPE-TC1001..TC1122, 122 IDs).
Los IDs P2 (TC001..TC089) NO están en este xlsx — sus fixes viven solo en
matriz_cases2.md y normalized-test-cases.json (commits previos).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
+++ b/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
@@ -1333,12 +1333,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1009 – E2E Alta de Viaje desde app pax para usuario app pax desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1009 – E2E Alta de Viaje desde app pax para usuario personal desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario personal desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1445,12 +1445,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1010 – E2E Alta de Viaje desde app pax para usuario app pax modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1010 – E2E Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1555,12 +1555,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1011 – E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1011 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1012 – E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1012 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1777,12 +1777,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1013 – E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1013 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1014 – E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1014 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -2002,12 +2002,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1015 – E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1015 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2114,12 +2114,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1016 – E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1016 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2230,12 +2230,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV001 – E2E Alta de Viaje para usuario app pax modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1017]</t>
+          <t>TS-STRIPE-TC-RV001 – E2E Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1017]</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -2329,12 +2329,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV002 – E2E Alta de Viaje para usuario app pax  desde app pax para usuario app pax modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1018]</t>
+          <t>TS-STRIPE-TC-RV002 – E2E Alta de Viaje para usuario personal  desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1018]</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax  desde app pax para usuario app pax modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje para usuario personal  desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -2428,12 +2428,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV003 – E2E Alta  de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1011]</t>
+          <t>TS-STRIPE-TC-RV003 – E2E Alta  de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1011]</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta  de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta  de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D20" s="6" t="n"/>
@@ -2527,12 +2527,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV004 – E2E Alta carrier de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1012]</t>
+          <t>TS-STRIPE-TC-RV004 – E2E Alta carrier de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1012]</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta carrier de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta carrier de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D21" s="6" t="n"/>
@@ -2626,12 +2626,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV005 – E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1013]</t>
+          <t>TS-STRIPE-TC-RV005 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1013]</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D22" s="6" t="n"/>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV006 – E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1014]</t>
+          <t>TS-STRIPE-TC-RV006 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1014]</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D23" s="6" t="n"/>
@@ -2824,12 +2824,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV007 – E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1015]</t>
+          <t>TS-STRIPE-TC-RV007 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1015]</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D24" s="6" t="n"/>
@@ -2923,12 +2923,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV008 – E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1016]</t>
+          <t>TS-STRIPE-TC-RV008 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1016]</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario app pax app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
@@ -3022,12 +3022,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1017 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1017 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -3132,12 +3132,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1018 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1018 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1019 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1019 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -3352,12 +3352,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1020 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1020 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -3462,12 +3462,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1021 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1021 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -3574,12 +3574,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1022 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1022 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3686,12 +3686,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1023 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1023 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3798,12 +3798,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1024 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1024 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3910,12 +3910,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1025 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1025 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1026 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1026 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1027 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1027 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -4240,12 +4240,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1028 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1028 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -4350,12 +4350,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1029 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1029 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -4462,12 +4462,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1030 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1030 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -4574,12 +4574,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1031 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1031 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -4686,12 +4686,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1032 – E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1032 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario app pax modo business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -6574,12 +6574,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1049 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1049 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1050 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1050 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -6794,12 +6794,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1051 — Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario app pax, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
+          <t>TS-STRIPE-TC1051 — Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario app pax, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
+          <t>Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
@@ -6904,12 +6904,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1052 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1052 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -7014,12 +7014,12 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1053 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1053 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -7126,12 +7126,12 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1054 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1054 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -7238,12 +7238,12 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1055 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1055 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -7350,12 +7350,12 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1056 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1056 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -7462,12 +7462,12 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1057 — Validar que al crear viaje desde carrier para usuario app pax con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
+          <t>TS-STRIPE-TC1057 — Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Validar que al crear viaje desde carrier para usuario app pax con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
+          <t>Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -7572,12 +7572,12 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1058 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1058 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -7682,12 +7682,12 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1059 — Validar que no se permite alta de viaje desde carrier para usuario app pax al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
+          <t>TS-STRIPE-TC1059 — Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Validar que no se permite alta de viaje desde carrier para usuario app pax al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
+          <t>Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -7792,12 +7792,12 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1060 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1060 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -7902,12 +7902,12 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1061 — Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario app pax, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
+          <t>TS-STRIPE-TC1061 — Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario app pax, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
+          <t>Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -8014,12 +8014,12 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1062 – E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1062 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -8126,12 +8126,12 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1063 — Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario app pax, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
+          <t>TS-STRIPE-TC1063 — Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario app pax, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
+          <t>Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -8238,12 +8238,12 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1064 — Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario app pax, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
+          <t>TS-STRIPE-TC1064 — Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario app pax, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
+          <t>Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -10126,12 +10126,12 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1081 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>TS-STRIPE-TC1081 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -10236,12 +10236,12 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1082 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>TS-STRIPE-TC1082 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -10347,12 +10347,12 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1083 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>TS-STRIPE-TC1083 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -10458,12 +10458,12 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1084 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>TS-STRIPE-TC1084 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -10569,12 +10569,12 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1085 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>TS-STRIPE-TC1085 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -10680,12 +10680,12 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1086 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>TS-STRIPE-TC1086 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -10791,12 +10791,12 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1087 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
+          <t>TS-STRIPE-TC1087 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
@@ -10902,12 +10902,12 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1088 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1088 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -11013,12 +11013,12 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1089 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1089 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr">
@@ -11124,12 +11124,12 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1090 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1090 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -11235,12 +11235,12 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1091 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1091 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
@@ -11346,12 +11346,12 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1092 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1092 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
@@ -11458,12 +11458,12 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1093 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1093 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
@@ -11571,12 +11571,12 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1094 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1094 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
@@ -11684,12 +11684,12 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1095 – E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>TS-STRIPE-TC1095 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario app pax con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">

</xml_diff>

<commit_message>
sync(xlsx): STRIPE_Test_Suite_Matriz_Sincronizado.xlsx reflejar matriz .md canónica (remover drift "E2E " y formato corto)
- 215 filas actualizadas en TEST_SUITE + TEST_SUITE 2.0 (184 con título canónico del md, 31 por normalización mecánica)
- Prefijo "E2E " eliminado: pre=347 → post=0
- Formato corto "Hold y Cobro desde App Driver" expandido a "Hold desde Alta de Viaje y Cobro desde App Driver": pre=146 → post=0
- Artefacto "app modo personal" limpiado
- Colapsado "desde app pax ... desde app pax" redundante
- Script sync-xlsx-canonical.py lee matriz_cases.md + matriz_cases2.md (incluye IDs TS-STRIPE-P2-TCxxx)
- openpyxl preserva estilos y colores
</commit_message>
<xml_diff>
--- a/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
+++ b/docs/gateway-pg/stripe/STRIPE_Test_Suite_Matriz_Sincronizado.xlsx
@@ -783,7 +783,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1002 – Validar vincular pasarela Stripe desde Magiis App Store con credenciales válidas y reflejar estado vinculado en UI y DBTS-STRIPE-TC003 – wallet validación -vinculalacion de eliminacion de tarjetas - tarjetas pre autorizadas - desde app pax</t>
+          <t>TS-STRIPE-TC1002 – Validar vincular pasarela Stripe desde Magiis App Store con credenciales válidas y reflejar estado vinculado en UI y DB</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1210,7 +1210,11 @@
           <t>TS-STRIPE-TC1006 – Validar exclusividad de pasarela activa e impedir vincular otro gateway mientras Stripe esté activo mostrando mensaje informativo</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Validar exclusividad de pasarela activa e impedir vincular otro gateway mientras Stripe esté activo mostrando mensaje informativo</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
@@ -1252,7 +1256,11 @@
           <t>TS-STRIPE-TC1007 – Validar persistencia de estado vinculado de Stripe tras recargar página y navegar entre secciones de Carrier</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Validar persistencia de estado vinculado de Stripe tras recargar página y navegar entre secciones de Carrier</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
@@ -1294,7 +1302,11 @@
           <t>TS-STRIPE-TC1008 – Validar que el request link y unlink de Stripe retorne status 200 y registre evento en logs o auditoría si aplica</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Validar que el request link y unlink de Stripe retorne status 200 y registre evento en logs o auditoría si aplica</t>
+        </is>
+      </c>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
@@ -1333,12 +1345,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1009 – E2E Alta de Viaje desde app pax para usuario personal desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1009 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario personal desde app pax modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1445,12 +1457,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1010 – E2E Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1010 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1555,12 +1567,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1011 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1011 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1665,12 +1677,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1012 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1012 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1777,12 +1789,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1013 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1013 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1889,12 +1901,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1014 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1014 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -2002,12 +2014,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1015 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1015 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2114,12 +2126,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1016 – E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1016 – Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2230,12 +2242,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV001 – E2E Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1017]</t>
+          <t>TS-STRIPE-TC-RV001 – Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1017]</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -2329,12 +2341,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV002 – E2E Alta de Viaje para usuario personal  desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1018]</t>
+          <t>TS-STRIPE-TC-RV002 – Alta de Viaje para usuario personal desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1018]</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal  desde app pax para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje para usuario personal desde app pax para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -2428,12 +2440,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV003 – E2E Alta  de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1011]</t>
+          <t>TS-STRIPE-TC-RV003 – Alta de Viaje para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1011]</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta  de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D20" s="6" t="n"/>
@@ -2527,12 +2539,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV004 – E2E Alta carrier de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1012]</t>
+          <t>TS-STRIPE-TC-RV004 – Alta carrier de Viaje para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1012]</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta carrier de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Alta carrier de Viaje para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D21" s="6" t="n"/>
@@ -2626,12 +2638,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV005 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1013]</t>
+          <t>TS-STRIPE-TC-RV005 – Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1013]</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D22" s="6" t="n"/>
@@ -2725,12 +2737,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV006 – E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1014]</t>
+          <t>TS-STRIPE-TC-RV006 – Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1014]</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal desde app pax con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje para usuario personal desde app pax con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D23" s="6" t="n"/>
@@ -2824,12 +2836,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV007 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1015]</t>
+          <t>TS-STRIPE-TC-RV007 – Alta de Viaje para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1015]</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D24" s="6" t="n"/>
@@ -2923,12 +2935,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC-RV008 – E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1016]</t>
+          <t>TS-STRIPE-TC-RV008 – Alta de Viaje para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS. [NOTA: variante exploratoria — misma combinación cubierta por TS-STRIPE-TC1016]</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje para usuario personal app modo personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
@@ -3022,12 +3034,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1017 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1017 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -3132,12 +3144,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1018 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1018 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -3242,12 +3254,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1019 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1019 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente (ID referenciable también como TS-STRIPE-TC1017-CARD-EXISTING)</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente (ID referenciable también como TS-STRIPE-TC1017-CARD-EXISTING)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -3352,12 +3364,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1020 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1020 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente (ID referenciable también como TS-STRIPE-TC1018-CARD-EXISTING)</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente (ID referenciable también como TS-STRIPE-TC1018-CARD-EXISTING)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -3462,12 +3474,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1021 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1021 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -3574,12 +3586,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1022 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1022 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -3686,12 +3698,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1023 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1023 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3798,12 +3810,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1024 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1024 – Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -3910,12 +3922,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1025 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1025 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -4020,12 +4032,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1026 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1026 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -4130,12 +4142,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1027 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1027 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -4240,12 +4252,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1028 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1028 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -4350,12 +4362,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1029 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1029 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -4462,12 +4474,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1030 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1030 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -4574,12 +4586,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1031 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1031 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -4686,12 +4698,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1032 – E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1032 – Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde app pax para usuario business con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -4798,12 +4810,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1033 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1033 – Validar vincular tarjeta y Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold (desde carrier) y Cobro desde App Driver — Vincular tarjeta nueva (seed)</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar vincular tarjeta y Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold (desde carrier) y Cobro desde App Driver — Vincular tarjeta nueva (seed)</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -4908,12 +4920,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1034 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1034 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -5018,12 +5030,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1035 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1035 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -5128,12 +5140,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1036 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1036 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -5238,12 +5250,12 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1037 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1037 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -5350,12 +5362,12 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1038 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1038 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -5462,12 +5474,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1039 — Validar que al crear viaje desde carrier con cliente contractor y pasajero app pax invitado usando tarjeta threeDSRequired con Hold ON, al fallar la autenticacion 3DS se muestra pop-up de error y la URL permanece en el formulario de alta sin crear el viaje</t>
+          <t>TS-STRIPE-TC1039 — Validar que al crear viaje desde carrier con cliente contractor y pasajero app pax invitado usando tarjeta threeDSRequired con Hold ON, al fallar la autenticación 3DS se muestra pop-up de error y la URL permanece en el formulario de alta sin crear el viaje</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Validar que al crear viaje desde carrier con cliente contractor y pasajero app pax invitado usando tarjeta threeDSRequired con Hold ON, al fallar la autenticacion 3DS se muestra pop-up de error y la URL permanece en el formulario de alta sin crear el viaje</t>
+          <t>Validar que al crear viaje desde carrier con cliente contractor y pasajero app pax invitado usando tarjeta threeDSRequired con Hold ON, al fallar la autenticación 3DS se muestra pop-up de error y la URL permanece en el formulario de alta sin crear el viaje</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -5574,12 +5586,12 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1040 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1040 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -5686,12 +5698,12 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1041 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1041 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -5796,12 +5808,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1042 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1042 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -5906,12 +5918,12 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1043 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1043 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
@@ -6016,12 +6028,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1044 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1044 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
@@ -6126,12 +6138,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1045 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1045 – Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
@@ -6238,12 +6250,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1046 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1046 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
@@ -6350,12 +6362,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1047 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1047 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
@@ -6462,12 +6474,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1048 – E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1048 – Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario colaborador o asociado de contractor con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
@@ -6574,12 +6586,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1049 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1049 – Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold ON — viaje pasa a estado "Buscando conductor" y aparece en columna "Por asignar" sin presentar modal 3DS</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold ON — viaje pasa a estado "Buscando conductor" y aparece en columna "Por asignar" sin presentar modal 3DS</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
@@ -6684,12 +6696,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1050 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1050 – Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — viaje pasa a estado "Buscando conductor" sin retención de fondos previa</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — viaje pasa a estado "Buscando conductor" sin retención de fondos previa</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -6794,12 +6806,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1051 — Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
+          <t>TS-STRIPE-TC1051 — Validar que en detalle del viaje aparece red flag "Validación 3DS pendiente" y botón "Reintentar autenticación" tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en "No autorizado" y viaje NO aparece en "Buscando conductor"</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Validar que en detalle del viaje aparece red flag Validacion 3DS pendiente y boton Reintentar autenticacion tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en No autorizado y viaje NO aparece en Buscando conductor</t>
+          <t>Validar que en detalle del viaje aparece red flag "Validación 3DS pendiente" y botón "Reintentar autenticación" tras fallo de 3DS — usuario personal, Hold ON, tarjeta fail3DS (4000 0000 0000 9235) — estado queda en "No autorizado" y viaje NO aparece en "Buscando conductor"</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
@@ -6904,12 +6916,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1052 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1052 – Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante origen/destino alternativo</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante origen/destino alternativo</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -7014,12 +7026,12 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1053 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1053 – Validar alta de viaje desde carrier para usuario personal con tarjeta success3DS (4000 0025 0000 3155) y Hold ON — modal 3DS se presenta, pasajero aprueba autenticación, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta success3DS (4000 0025 0000 3155) y Hold ON — modal 3DS se presenta, pasajero aprueba autenticación, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -7126,12 +7138,12 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1054 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1054 – Validar alta de viaje desde carrier para usuario personal con tarjeta success3DS (4000 0025 0000 3155) y Hold OFF — modal 3DS se presenta, pasajero aprueba autenticación, viaje pasa a "Buscando conductor" sin retención previa</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta success3DS (4000 0025 0000 3155) y Hold OFF — modal 3DS se presenta, pasajero aprueba autenticación, viaje pasa a "Buscando conductor" sin retención previa</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -7238,12 +7250,12 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1055 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1055 – Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold ON — 3DS forzado en todas las transacciones, autenticación exitosa, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold ON — 3DS forzado en todas las transacciones, autenticación exitosa, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -7350,12 +7362,12 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1056 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1056 – Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold OFF — 3DS forzado, autenticación exitosa, viaje activo sin hold</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold OFF — 3DS forzado, autenticación exitosa, viaje activo sin hold</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -7462,12 +7474,12 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1057 — Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
+          <t>TS-STRIPE-TC1057 — Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticación aparece pop-up de error y el viaje queda en estado "No autorizado" sin pasar a "Por asignar"</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticacion aparece pop-up de error y el viaje queda en estado No autorizado sin pasar a Por asignar</t>
+          <t>Validar que al crear viaje desde carrier para usuario personal con tarjeta fail3DS (4000 0000 0000 9235) y Hold ON se presenta modal 3DS, al fallar la autenticación aparece pop-up de error y el viaje queda en estado "No autorizado" sin pasar a "Por asignar"</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -7572,12 +7584,12 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1058 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1058 – Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante set 2</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante set 2</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -7682,12 +7694,12 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1059 — Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
+          <t>TS-STRIPE-TC1059 — Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinación y el viaje no se crea</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinacion y el viaje no se crea</t>
+          <t>Validar que no se permite alta de viaje desde carrier para usuario personal al intentar vincular tarjeta con fondos insuficientes (4000 0000 0000 9995) con Hold ON — sistema muestra error de declinación y el viaje no se crea</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -7792,12 +7804,12 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1060 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1060 – Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante set 2 alternativo</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta preautorizada exitosa (4242 4242 4242 4242) con Hold OFF — variante set 2 alternativo</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -7902,12 +7914,12 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1061 — Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
+          <t>TS-STRIPE-TC1061 — Validar reintento exitoso de autenticación 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso con success3DS — viaje pasa a "Buscando conductor", red flag y botón "Reintentar" desaparecen</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Validar reintento exitoso de autenticacion 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso — viaje pasa a Buscando conductor, red flag y boton Reintentar desaparecen</t>
+          <t>Validar reintento exitoso de autenticación 3DS desde detalle del viaje — usuario personal, Hold ON, fallo inicial con fail3DS (4000 0000 0000 9235), reintento exitoso con success3DS — viaje pasa a "Buscando conductor", red flag y botón "Reintentar" desaparecen</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -8014,12 +8026,12 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1062 – E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1062 – Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold OFF — variante set 2</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario personal con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar alta de viaje desde carrier para usuario personal con tarjeta always_authenticate (4000 0027 6000 3184) y Hold OFF — variante set 2</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -8126,12 +8138,12 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1063 — Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
+          <t>TS-STRIPE-TC1063 — Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — selección de tarjeta guardada, reintento de hold exitoso, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — seleccion de tarjeta guardada, reintento de hold exitoso, viaje pasa a Buscando conductor (PENDIENTE: requiere payment-method component en travel-detail)</t>
+          <t>Validar cambio a tarjeta vinculada existente desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — selección de tarjeta guardada, reintento de hold exitoso, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -8238,12 +8250,12 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1064 — Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
+          <t>TS-STRIPE-TC1064 — Validar vinculación de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Validar vinculacion de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a Buscando conductor (PENDIENTE: requiere flujo de vinculacion en travel-detail)</t>
+          <t>Validar vinculación de tarjeta nueva desde detalle del viaje tras fallo 3DS — usuario personal, Hold ON — nueva tarjeta success3DS (4000 0025 0000 3155), 3DS aprobado, viaje pasa a "Buscando conductor"</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -8350,12 +8362,12 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1065 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1065 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -8460,12 +8472,12 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1066 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1066 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -8570,12 +8582,12 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1067 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1067 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -8680,12 +8692,12 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1068 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1068 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -8790,12 +8802,12 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1069 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1069 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -8902,12 +8914,12 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1070 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1070 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Vincular tarjeta nueva</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -9014,12 +9026,12 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1071 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1071 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -9126,12 +9138,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1072 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1072 – Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Validar Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS — Usar tarjeta vinculada existente</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -9238,12 +9250,12 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1073 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1073 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -9348,12 +9360,12 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1074 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>TS-STRIPE-TC1074 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -9458,12 +9470,12 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1075 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1075 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -9568,12 +9580,12 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1076 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>TS-STRIPE-TC1076 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver.</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -9678,12 +9690,12 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1077 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1077 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
@@ -9790,12 +9802,12 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1078 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1078 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -9902,12 +9914,12 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1079 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1079 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
@@ -10014,12 +10026,12 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1080 – E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>TS-STRIPE-TC1080 – Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold y Cobro desde App Driver con validacion 3DS.</t>
+          <t>Alta de Viaje desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validacion 3DS.</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -10126,12 +10138,12 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1081 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>TS-STRIPE-TC1081 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -10236,12 +10248,12 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1082 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>TS-STRIPE-TC1082 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -10347,12 +10359,12 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1083 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>TS-STRIPE-TC1083 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -10458,12 +10470,12 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1084 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>TS-STRIPE-TC1084 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -10569,12 +10581,12 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1085 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>TS-STRIPE-TC1085 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -10680,12 +10692,12 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1086 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>TS-STRIPE-TC1086 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -10791,12 +10803,12 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1087 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
+          <t>TS-STRIPE-TC1087 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - Prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
@@ -10902,12 +10914,12 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1088 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1088 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -11013,12 +11025,12 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1089 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1089 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr">
@@ -11124,12 +11136,12 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1090 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1090 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -11235,12 +11247,12 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1091 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1091 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
@@ -11346,12 +11358,12 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1092 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1092 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago exitoso con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago exitoso con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
@@ -11458,12 +11470,12 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1093 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1093 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago rechazado con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – pago rechazado con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
@@ -11571,12 +11583,12 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1094 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1094 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – error con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – error con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
@@ -11684,12 +11696,12 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1095 – E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>TS-STRIPE-TC1095 – Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla 3D Secure</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario personal con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>Validar Alta de viaje desde carrier para usuario personal – cargo a bordo – falla 3D Secure</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">
@@ -11797,12 +11809,12 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1096 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>TS-STRIPE-TC1096 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
@@ -11907,12 +11919,12 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1097 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>TS-STRIPE-TC1097 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
@@ -12018,12 +12030,12 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1098 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>TS-STRIPE-TC1098 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
@@ -12129,12 +12141,12 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1099 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>TS-STRIPE-TC1099 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
@@ -12240,12 +12252,12 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1100 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>TS-STRIPE-TC1100 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
@@ -12351,12 +12363,12 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1101 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>TS-STRIPE-TC1101 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -12462,12 +12474,12 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1102 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1102 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -12573,12 +12585,12 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1103 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1103 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
@@ -12684,12 +12696,12 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1104 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1104 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -12795,12 +12807,12 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1105 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1105 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -12906,12 +12918,12 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1106 – E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1106 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -13017,12 +13029,12 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1107 – E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1107 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago exitoso con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago exitoso con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
@@ -13129,12 +13141,12 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1108 – E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1108 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago rechazado con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Pago rechazado con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – pago rechazado con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -13242,12 +13254,12 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1109 – E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>TS-STRIPE-TC1109 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – error con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla Error con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – error con 3D Secure obligatorio</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
@@ -13355,12 +13367,12 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1110 – E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>TS-STRIPE-TC1110 – Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla 3D Secure</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario usuario colaborador o asociado de contractor con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla 3D Secure.</t>
+          <t>Validar Alta de viaje desde carrier para usuario colaborador o asociado de contractor – cargo a bordo – falla 3D Secure</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -13468,12 +13480,12 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1111 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>TS-STRIPE-TC1111 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con pago exitoso.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – pago exitoso</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -13578,12 +13590,12 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1112 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>TS-STRIPE-TC1112 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con pago rechazado genérico.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – pago rechazado genérico</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -13689,12 +13701,12 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1113 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>TS-STRIPE-TC1113 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por fondos insuficientes.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – fondos insuficientes</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -13800,12 +13812,12 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1114 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>TS-STRIPE-TC1114 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por ser una tarjeta reportada como perdida.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta reportada como perdida</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
@@ -13911,12 +13923,12 @@
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1115 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>TS-STRIPE-TC1115 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por CVC incorrecto.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – CVC incorrecto</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
@@ -14022,12 +14034,12 @@
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1116 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>TS-STRIPE-TC1116 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por por tratarse de una tarjeta robada.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta robada</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
@@ -14133,12 +14145,12 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1117 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1117 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del CVC - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – falla comprobación CVC (antifraude)</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
@@ -14244,12 +14256,12 @@
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1118 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1118 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Riesgo Maximo - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – riesgo máximo (antifraude)</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
@@ -14355,12 +14367,12 @@
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1119 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1119 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por tarjeta siempre bloqueada - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – tarjeta siempre bloqueada (antifraude)</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
@@ -14466,12 +14478,12 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1120 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1120 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación del código postal con riesgo elevado - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – falla código postal con riesgo elevado (antifraude)</t>
         </is>
       </c>
       <c r="D129" s="6" t="inlineStr">
@@ -14577,12 +14589,12 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1121 – E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>TS-STRIPE-TC1121 – Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago rechazado por Falla la comprobación Dirección no disponible - prevención antifraude.</t>
+          <t>Validar Alta de viaje desde carrier para usuario empresa individuo – cargo a bordo – dirección no disponible (antifraude)</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -14688,12 +14700,12 @@
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>TS-STRIPE-TC1122 – E</t>
+          <t>TS-STRIPE-TC1122 – Validar validar eliminar satisfactoriamente desde wallet tarjeta previamente vinculada con validación 3D Secure desde app pax para usuario personal</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>E2E Alta de viaje desde carrier para usuario empresa individuo con cobro de tarjeta de crédito - cargo a Bordo con Pago exitoso con tarjeta con 3D secure obligatorio.</t>
+          <t>Validar validar eliminar satisfactoriamente desde wallet tarjeta previamente vinculada con validación 3D Secure desde app pax para usuario personal</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -15214,12 +15226,12 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC001 – Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC001 – Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -15333,12 +15345,12 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC002 – Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC002 – Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -15452,12 +15464,12 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC003 – Validar E2E selección de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC003 – Validar selección de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -15570,12 +15582,12 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC004 – Validar E2E selección de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC004 – Validar selección de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -15688,12 +15700,12 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC005 – Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC005 – Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -15807,12 +15819,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC006 – Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC006 – Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje desde App PAX para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -15926,12 +15938,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC007 – Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC007 – Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -16045,12 +16057,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC008 – Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC008 – Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -16164,12 +16176,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC009 – Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC009 – Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -16283,12 +16295,12 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC010 – Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC010 – Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario sin datos filiatorios vinculado a pasajero existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -16402,12 +16414,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC011 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC011 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -16521,12 +16533,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC012 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC012 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -16640,12 +16652,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC013 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC013 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -16759,12 +16771,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC014 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC014 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -16878,12 +16890,12 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC015 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC015 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -16997,12 +17009,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC016 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC016 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -17116,12 +17128,12 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC017 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC017 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -17235,12 +17247,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC018 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC018 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario colaborador existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -17354,12 +17366,12 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC019 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC019 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -17473,12 +17485,12 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC020 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC020 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -17592,12 +17604,12 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC021 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC021 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -17711,12 +17723,12 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC022 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC022 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -17830,12 +17842,12 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC023 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC023 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -17949,12 +17961,12 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC024 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC024 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -18068,12 +18080,12 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC025 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC025 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -18187,12 +18199,12 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC026 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC026 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario app pax existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario personal existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -18306,12 +18318,12 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC027 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC027 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -18425,12 +18437,12 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC028 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC028 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -18544,12 +18556,12 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC029 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC029 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -18663,12 +18675,12 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC030 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC030 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -18782,12 +18794,12 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC031 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC031 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -18901,12 +18913,12 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC032 – Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC032 – Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con número de teléfono vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -19020,12 +19032,12 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC033 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC033 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -19139,12 +19151,12 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC034 – Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>TS-STRIPE-P2-TC034 – Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E alta de viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3D secure</t>
+          <t>Validar Alta de Viaje desde Quote para usuario con mail vinculado a usuario empresa individuo existente con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3D Secure</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -19258,12 +19270,12 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC035 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC035 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -19378,12 +19390,12 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC036 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC036 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -19498,12 +19510,12 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC037 – Validar E2E selección de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC037 – Validar selección de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -19618,12 +19630,12 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC038 – Validar E2E selección de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC038 – Validar selección de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -19738,12 +19750,12 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC039 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC039 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -19858,12 +19870,12 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC040 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC040 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde portal Contractor para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde portal contractor para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -19978,12 +19990,12 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC041 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC041 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -20097,12 +20109,12 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC042 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC042 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -20216,12 +20228,12 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC043 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC043 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -20335,12 +20347,12 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC044 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC044 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -20454,12 +20466,12 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC045 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC045 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -20573,12 +20585,12 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC046 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC046 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario colaborador con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -20692,12 +20704,12 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC047 – Validar E2E vinculación y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada y edición de fechas para validar consistencia de datos y finalización desde App Driver</t>
+          <t>TS-STRIPE-P2-TC047 – Validar vinculación y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada y edición de fechas para validar consistencia de datos y finalización desde App Driver</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada y edición de fechas para validar consistencia de datos y finalización desde App Driver</t>
+          <t>Validar vinculación y alta de viaje recurrente desde Carrier para usuario colaborador de contractor con tarjeta preautorizada y edición de fechas para validar consistencia de datos y finalización desde App Driver</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -20811,12 +20823,12 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC048 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC048 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -20930,12 +20942,12 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC049 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC049 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -21049,12 +21061,12 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC050 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC050 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -21168,12 +21180,12 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC051 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC051 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -21287,12 +21299,12 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC052 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC052 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -21406,12 +21418,12 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC053 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC053 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario app pax de contractor con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario personal con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -21525,12 +21537,12 @@
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC054 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC054 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -21644,12 +21656,12 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC055 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC055 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -21763,12 +21775,12 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC056 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC056 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -21882,12 +21894,12 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC057 – Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>TS-STRIPE-P2-TC057 – Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E selección de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver</t>
+          <t>Validar selección de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -22001,12 +22013,12 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC058 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC058 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
@@ -22120,12 +22132,12 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC059 – Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC059 – Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Validar E2E vinculación de tarjeta y alta de viaje recurrente desde Carrier para usuario empresa individuo con tarjeta preautorizada sin hold y cobro desde App Driver con validación 3DS</t>
+          <t>Validar vinculación de tarjeta y Alta de Viaje Recurrente desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -22244,7 +22256,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22261,7 +22273,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22278,7 +22290,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22295,7 +22307,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22312,7 +22324,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Reactivación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22329,7 +22341,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Reactivación de viaje cancelado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22346,7 +22358,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22363,7 +22375,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22380,7 +22392,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22397,7 +22409,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22414,7 +22426,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Clonación de viaje cancelado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22431,7 +22443,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Clonación de viaje cancelado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22448,7 +22460,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22465,7 +22477,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22482,7 +22494,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22499,7 +22511,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22516,7 +22528,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22533,7 +22545,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22550,7 +22562,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22567,7 +22579,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22584,7 +22596,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22601,7 +22613,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22613,12 +22625,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC082 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC082 – Validar Edición de viaje programado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Edición de viaje programado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22630,12 +22642,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC083 – Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC083 – Validar Edición de viaje programado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Edición de viaje programado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22652,7 +22664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22669,7 +22681,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Vincular tarjeta nueva</t>
         </is>
       </c>
     </row>
@@ -22686,7 +22698,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22703,7 +22715,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>Validar Alta de viaje y edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver — Usar tarjeta vinculada existente</t>
         </is>
       </c>
     </row>
@@ -22715,12 +22727,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC088 – Validar Clonación de viaje finalizado desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC088 – Validar Edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Edición en conflicto desde carrier para usuario empresa individuo con Tarjeta Preautorizada Hold desde Alta de Viaje y Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>
@@ -22732,12 +22744,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TS-STRIPE-P2-TC089 – Validar Clonación de viaje finalizado para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
+          <t>TS-STRIPE-P2-TC089 – Validar Edición en conflicto para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>Validar Edición en conflicto para usuario empresa individuo con Tarjeta Preautorizada sin Hold desde Alta de Viaje, Cobro desde App Driver con validación 3DS</t>
         </is>
       </c>
     </row>

</xml_diff>